<commit_message>
Confrontar 39 evidências e corrigir Word e figuras da Seção 1
Explicita restrições, derivações e inferências; confere Driesse e a proveniência PVDAQ. Acrescenta seis verificações de relações físicas e geração de DOCX/PDF no notebook com dez células executadas por IPython. Corrige os seis slides com fundo preto e PNGs de compatibilidade válidos, preservando os demais autores. Não repete a bibliometria nem publica PDFs integrais de terceiros.
</commit_message>
<xml_diff>
--- a/secoes/01_Recurso_Solar/producao/bibliografia/Matriz_Corpus_e_Curadoria_Secao_01.xlsx
+++ b/secoes/01_Recurso_Solar/producao/bibliografia/Matriz_Corpus_e_Curadoria_Secao_01.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visao_Geral" sheetId="1" r:id="R15ec1164c7a7460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_1" sheetId="2" r:id="Ra70f4cb01f814d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_2" sheetId="3" r:id="Rf61dd4a6f9b24ec7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_3" sheetId="4" r:id="R0d1b1eb12faa48f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_4" sheetId="5" r:id="Rf0379c4128854dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa_Corpus" sheetId="6" r:id="R1bb37e957f924942"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracao_Semantica" sheetId="7" r:id="R92bacfa978444288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendencias" sheetId="8" r:id="Ra1727fd046e84864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selecao_Critica" sheetId="9" r:id="R39ac887636c84170"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visao_Geral" sheetId="1" r:id="R74b0fc6f5ce04ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_1" sheetId="2" r:id="R6e7c5e5cea9e4066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_2" sheetId="3" r:id="R83480ecb51214b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_3" sheetId="4" r:id="R5b530f4fadd04edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus_1_4" sheetId="5" r:id="R4d068d7bae514acc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa_Corpus" sheetId="6" r:id="R73294078225d435c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracao_Semantica" sheetId="7" r:id="R4e1e238481124250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendencias" sheetId="8" r:id="R3cb4c939524c437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selecao_Critica" sheetId="9" r:id="R83d1bcc7dbcd43af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confronto_Cientifico" sheetId="10" r:id="R0677f4761ba84794"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -148,6 +149,27 @@
     <x:tableColumn id="7" name="Contribuição"/>
     <x:tableColumn id="8" name="Limites e pendências"/>
     <x:tableColumn id="9" name="Fonte"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ConfrontoCientifico" displayName="ConfrontoCientifico" ref="A1:M40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Subseção"/>
+    <x:tableColumn id="3" name="Fonte"/>
+    <x:tableColumn id="4" name="Página PDF"/>
+    <x:tableColumn id="5" name="Página impressa"/>
+    <x:tableColumn id="6" name="Afirmação analisada"/>
+    <x:tableColumn id="7" name="Classificação"/>
+    <x:tableColumn id="8" name="Justificativa científica"/>
+    <x:tableColumn id="9" name="Confronto entre fontes"/>
+    <x:tableColumn id="10" name="Consequência editorial"/>
+    <x:tableColumn id="11" name="Âncora conferida"/>
+    <x:tableColumn id="12" name="SHA-256 arquivo"/>
+    <x:tableColumn id="13" name="SHA-256 página"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -393,7 +415,7 @@
         <x:v>https://drive.google.com/drive/folders/1HTae6qXkmgPfNiTsWfdtKFiXvHUBSrjl</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Evidências localizadas e manuscrito revisado</x:v>
+        <x:v>Afirmações confrontadas; manuscrito e seis slides revisados</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="56" customHeight="1">
@@ -413,7 +435,7 @@
         <x:v>https://drive.google.com/drive/folders/19h7iXMeNxiQdDMlKUj6MXYEGeBm4tM3x</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Redação fundamentada; leituras complementares pendentes</x:v>
+        <x:v>Afirmações confrontadas; limites e derivações explicitados</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="56" customHeight="1">
@@ -433,7 +455,7 @@
         <x:v>https://drive.google.com/drive/folders/1jQKp0Saama6K7r8ITLeNlILSsAdtUi8r</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Redação fundamentada; leituras complementares pendentes</x:v>
+        <x:v>Afirmações confrontadas; inferências explicitadas</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="56" customHeight="1">
@@ -453,7 +475,7 @@
         <x:v>https://drive.google.com/drive/folders/15skeLT9fZ5zsiON3JRCDa28kujinwvJz</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
-        <x:v>Redação fundamentada; leituras complementares pendentes</x:v>
+        <x:v>Afirmações confrontadas; medição e incerteza delimitadas</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -506,6 +528,1673 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="68" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="85" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="85" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="85" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="58" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="75" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="48" customHeight="1">
+      <x:c r="A1" s="14" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B1" s="14" t="str">
+        <x:v>Subseção</x:v>
+      </x:c>
+      <x:c r="C1" s="14" t="str">
+        <x:v>Fonte</x:v>
+      </x:c>
+      <x:c r="D1" s="14" t="str">
+        <x:v>Página PDF</x:v>
+      </x:c>
+      <x:c r="E1" s="14" t="str">
+        <x:v>Página impressa</x:v>
+      </x:c>
+      <x:c r="F1" s="14" t="str">
+        <x:v>Afirmação analisada</x:v>
+      </x:c>
+      <x:c r="G1" s="14" t="str">
+        <x:v>Classificação</x:v>
+      </x:c>
+      <x:c r="H1" s="14" t="str">
+        <x:v>Justificativa científica</x:v>
+      </x:c>
+      <x:c r="I1" s="14" t="str">
+        <x:v>Confronto entre fontes</x:v>
+      </x:c>
+      <x:c r="J1" s="14" t="str">
+        <x:v>Consequência editorial</x:v>
+      </x:c>
+      <x:c r="K1" s="14" t="str">
+        <x:v>Âncora conferida</x:v>
+      </x:c>
+      <x:c r="L1" s="14" t="str">
+        <x:v>SHA-256 arquivo</x:v>
+      </x:c>
+      <x:c r="M1" s="14" t="str">
+        <x:v>SHA-256 página</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="50.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A2" s="13" t="str">
+        <x:v>EV001</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C2" s="13" t="str">
+        <x:v>B12</x:v>
+      </x:c>
+      <x:c r="D2" s="13" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E2" s="13" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F2" s="13" t="str">
+        <x:v>A distância Terra–Sol modifica a irradiância extraterrestre normal.</x:v>
+      </x:c>
+      <x:c r="G2" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H2" s="13" t="str">
+        <x:v>A p. 9 vincula a variação orbital à irradiância normal. A equação 1.4.1b do exemplar imprime 0,00719; o código pvlib 0.16.1 imprime 0,000719. Há divergência documental real, conferida também na imagem da página.</x:v>
+      </x:c>
+      <x:c r="I2" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J2" s="13" t="str">
+        <x:v>Manter 0,000719 para reproduzir a implementação e registrar a divergência; não reproduzir o coeficiente do livro como se fosse o executado.</x:v>
+      </x:c>
+      <x:c r="K2" s="13" t="str">
+        <x:v>Variation of the earth-sun distance</x:v>
+      </x:c>
+      <x:c r="L2" s="13" t="str">
+        <x:v>db6ac445398a88a7670cbee02db18c426732e8104ee56e4cfb81fa86be85f4da</x:v>
+      </x:c>
+      <x:c r="M2" s="13" t="str">
+        <x:v>dd58eae18e88641d0cb36166491ac419dd4102d7b5423658288547689bba56b0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A3" s="13" t="str">
+        <x:v>EV002</x:v>
+      </x:c>
+      <x:c r="B3" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C3" s="13" t="str">
+        <x:v>B12</x:v>
+      </x:c>
+      <x:c r="D3" s="13" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E3" s="13" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="str">
+        <x:v>Zenital é contado desde a vertical; elevação é seu complemento.</x:v>
+      </x:c>
+      <x:c r="G3" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H3" s="13" t="str">
+        <x:v>As definições de zenital e elevação são explícitas na p. 13. A elevação complementa o zenital no mesmo referencial geométrico.</x:v>
+      </x:c>
+      <x:c r="I3" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J3" s="13" t="str">
+        <x:v>Identificar zenital geométrico no esquema; não confundir com o ângulo de incidência em superfície inclinada.</x:v>
+      </x:c>
+      <x:c r="K3" s="13" t="str">
+        <x:v>the angle between the vertical and the line to the sun</x:v>
+      </x:c>
+      <x:c r="L3" s="13" t="str">
+        <x:v>db6ac445398a88a7670cbee02db18c426732e8104ee56e4cfb81fa86be85f4da</x:v>
+      </x:c>
+      <x:c r="M3" s="13" t="str">
+        <x:v>ae9319c24d2de1eaef3fe3f89c9e28692ca0558366f88a3b8c9cf451f67662ac</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A4" s="13" t="str">
+        <x:v>EV003</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="str">
+        <x:v>B12</x:v>
+      </x:c>
+      <x:c r="D4" s="13" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="str">
+        <x:v>A relação esférica liga latitude, declinação e ângulo horário ao zenital.</x:v>
+      </x:c>
+      <x:c r="G4" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="str">
+        <x:v>A equação 1.6.5, p. 15, resulta de inclinação zero e coincide com a relação apresentada. O SPA acrescenta correções astronômicas/topocêntricas.</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="str">
+        <x:v>Manter a equação esférica como fundamento; não apresentá-la como descrição integral do SPA.</x:v>
+      </x:c>
+      <x:c r="K4" s="13" t="str">
+        <x:v>the angle of incidence is the zenith angle</x:v>
+      </x:c>
+      <x:c r="L4" s="13" t="str">
+        <x:v>db6ac445398a88a7670cbee02db18c426732e8104ee56e4cfb81fa86be85f4da</x:v>
+      </x:c>
+      <x:c r="M4" s="13" t="str">
+        <x:v>00f1d5902f966554939cec8111a62fb0ccec88cd43c18e5ceee57e29c2633cbb</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A5" s="13" t="str">
+        <x:v>EV004</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="str">
+        <x:v>B12</x:v>
+      </x:c>
+      <x:c r="D5" s="13" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E5" s="13" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="str">
+        <x:v>O livro adota origem azimutal no sul, com sinais distintos da convenção SPA.</x:v>
+      </x:c>
+      <x:c r="G5" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H5" s="13" t="str">
+        <x:v>Duffie usa origem no sul. Reda/Andreas usa norte e sentido horário; as convenções não são intercambiáveis sem conversão.</x:v>
+      </x:c>
+      <x:c r="I5" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J5" s="13" t="str">
+        <x:v>Usar A_s para o azimute adotado e explicitar A_s=(gamma_s+180 graus) mod 360 graus; no zênite a projeção horizontal e o azimute são indefinidos.</x:v>
+      </x:c>
+      <x:c r="K5" s="13" t="str">
+        <x:v>east of south are negative</x:v>
+      </x:c>
+      <x:c r="L5" s="13" t="str">
+        <x:v>db6ac445398a88a7670cbee02db18c426732e8104ee56e4cfb81fa86be85f4da</x:v>
+      </x:c>
+      <x:c r="M5" s="13" t="str">
+        <x:v>ae9319c24d2de1eaef3fe3f89c9e28692ca0558366f88a3b8c9cf451f67662ac</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>EV005</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="str">
+        <x:v>B12</x:v>
+      </x:c>
+      <x:c r="D6" s="13" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E6" s="13" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="str">
+        <x:v>Ao nível do mar, a aproximação secante da massa de ar é apresentada para zenitais até cerca de 70°.</x:v>
+      </x:c>
+      <x:c r="G6" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H6" s="13" t="str">
+        <x:v>A p. 9 limita explicitamente a aproximação secante a 0–70 graus e ao nível do mar; a p. 10 discute a curvatura terrestre para zenitais maiores.</x:v>
+      </x:c>
+      <x:c r="I6" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J6" s="13" t="str">
+        <x:v>Acrescentar nível do mar ao domínio didático. Distinguir massa relativa e correção de pressão; não extrapolar a secante ao horizonte.</x:v>
+      </x:c>
+      <x:c r="K6" s="13" t="str">
+        <x:v>at sea level</x:v>
+      </x:c>
+      <x:c r="L6" s="13" t="str">
+        <x:v>db6ac445398a88a7670cbee02db18c426732e8104ee56e4cfb81fa86be85f4da</x:v>
+      </x:c>
+      <x:c r="M6" s="13" t="str">
+        <x:v>dd58eae18e88641d0cb36166491ac419dd4102d7b5423658288547689bba56b0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="13" t="str">
+        <x:v>EV006</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="str">
+        <x:v>B23</x:v>
+      </x:c>
+      <x:c r="D7" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="13" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F7" s="13" t="str">
+        <x:v>O tempo solar verdadeiro depende de longitude, fuso e equação do tempo.</x:v>
+      </x:c>
+      <x:c r="G7" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H7" s="13" t="str">
+        <x:v>NOAA relaciona tempo solar verdadeiro, equação do tempo, longitude e fuso. É uma aproximação diferente do SPA e usa 366 no ano bissexto.</x:v>
+      </x:c>
+      <x:c r="I7" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J7" s="13" t="str">
+        <x:v>Usar NOAA apenas como explicação do tempo solar; manter o denominador 365 do Spencer executado e não fundir os dois procedimentos.</x:v>
+      </x:c>
+      <x:c r="K7" s="13" t="str">
+        <x:v>the true solar time</x:v>
+      </x:c>
+      <x:c r="L7" s="13" t="str">
+        <x:v>7fa1fdb5f6b5c05ab1ec3ffde92e6fb2d5df98bf1a87055075ae2c3c1240a627</x:v>
+      </x:c>
+      <x:c r="M7" s="13" t="str">
+        <x:v>93ff8495c12d032fabc84a6683b5f7a42aed69d33e56e27f8b2ea476ddbb27c4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="13" t="str">
+        <x:v>EV007</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C8" s="13" t="str">
+        <x:v>B23</x:v>
+      </x:c>
+      <x:c r="D8" s="13" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E8" s="13" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F8" s="13" t="str">
+        <x:v>O critério de nascer e pôr do Sol em 90,833° inclui aproximações de refração e tamanho angular do disco solar.</x:v>
+      </x:c>
+      <x:c r="G8" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H8" s="13" t="str">
+        <x:v>NOAA fixa 90,833 graus para nascer/pôr, combinando refração e tamanho do disco. Esse limiar não é o horizonte geométrico do centro solar.</x:v>
+      </x:c>
+      <x:c r="I8" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J8" s="13" t="str">
+        <x:v>Explicitar disco solar e refração; manter max(0,cos zenital) como convenção geométrica do cálculo extraterrestre.</x:v>
+      </x:c>
+      <x:c r="K8" s="13" t="str">
+        <x:v>size of the solar disk</x:v>
+      </x:c>
+      <x:c r="L8" s="13" t="str">
+        <x:v>7fa1fdb5f6b5c05ab1ec3ffde92e6fb2d5df98bf1a87055075ae2c3c1240a627</x:v>
+      </x:c>
+      <x:c r="M8" s="13" t="str">
+        <x:v>9788c950e1aded2709fb57da7909dfd40792dd060ce35c34918e6ef4ed992a38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="13" t="str">
+        <x:v>EV008</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="str">
+        <x:v>B31</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="13" t="str">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="F9" s="13" t="str">
+        <x:v>O artigo SPA explicita azimute desde o norte e longitude positiva para leste.</x:v>
+      </x:c>
+      <x:c r="G9" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H9" s="13" t="str">
+        <x:v>O resumo do artigo informa a mudança de origem azimutal e longitude positiva para leste.</x:v>
+      </x:c>
+      <x:c r="I9" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J9" s="13" t="str">
+        <x:v>Conservar norte 0 graus e sentido horário em figuras, código, configurações e texto.</x:v>
+      </x:c>
+      <x:c r="K9" s="13" t="str">
+        <x:v>measured from north and eastward</x:v>
+      </x:c>
+      <x:c r="L9" s="13" t="str">
+        <x:v>e1a6603e2a5fa169b77b7e4f9468323d73e67af7175e3e043d58b79b25087105</x:v>
+      </x:c>
+      <x:c r="M9" s="13" t="str">
+        <x:v>f3439aecbac80986ab4dc03814d399785b3ac007f667e3191d62a158a919edc4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="13" t="str">
+        <x:v>EV009</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="str">
+        <x:v>B31</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E10" s="13" t="str">
+        <x:v>578</x:v>
+      </x:c>
+      <x:c r="F10" s="13" t="str">
+        <x:v>A precisão angular atribuída ao SPA se refere ao cálculo de posição solar.</x:v>
+      </x:c>
+      <x:c r="G10" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H10" s="13" t="str">
+        <x:v>A p. 578 atribui incerteza angular ao SPA e explicita sensibilidade às escalas de tempo e DUT1. Não é uma avaliação do sensor PVDAQ.</x:v>
+      </x:c>
+      <x:c r="I10" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J10" s="13" t="str">
+        <x:v>Não transferir a incerteza publicada do algoritmo ao sensor, à irradiância nem ao caso com entradas padrão.</x:v>
+      </x:c>
+      <x:c r="K10" s="13" t="str">
+        <x:v>In this report we describe a procedure</x:v>
+      </x:c>
+      <x:c r="L10" s="13" t="str">
+        <x:v>e1a6603e2a5fa169b77b7e4f9468323d73e67af7175e3e043d58b79b25087105</x:v>
+      </x:c>
+      <x:c r="M10" s="13" t="str">
+        <x:v>96c32b1720a9a922ae08adc5f899d1706a99572c314b50a70dfbeccfe5c432d8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A11" s="13" t="str">
+        <x:v>EV010</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>B32</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F11" s="13" t="str">
+        <x:v>O tratamento topocêntrico distingue elevação sem e com refração.</x:v>
+      </x:c>
+      <x:c r="G11" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H11" s="13" t="str">
+        <x:v>As equações 41–44, pp. 10–11, separam elevação sem refração, correção dependente de pressão/temperatura e elevação corrigida.</x:v>
+      </x:c>
+      <x:c r="I11" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J11" s="13" t="str">
+        <x:v>Manter zenital geométrico na projeção extraterrestre e declarar zenital aparente no cálculo de incidência adotado no projeto.</x:v>
+      </x:c>
+      <x:c r="K11" s="13" t="str">
+        <x:v>without atmospheric refraction correction</x:v>
+      </x:c>
+      <x:c r="L11" s="13" t="str">
+        <x:v>1b9e2b6131d89ebc17fe4c047e64a0168143c949bfe6fafe06d856d651555cc2</x:v>
+      </x:c>
+      <x:c r="M11" s="13" t="str">
+        <x:v>ea84c8fd306b34a548e333e16eabe5ead637179e16dc229f134c1ac94b82e383</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A12" s="13" t="str">
+        <x:v>EV011</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>B32</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>A-15</x:v>
+      </x:c>
+      <x:c r="F12" s="13" t="str">
+        <x:v>O exemplo numérico informa data, fuso, localização, pressão, altitude, temperatura e ΔT.</x:v>
+      </x:c>
+      <x:c r="G12" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H12" s="13" t="str">
+        <x:v>O exemplo A.5, p. A-15, fornece todos os parâmetros usados no teste, incluindo fuso fixo -7, pressão 820 mbar e deltaT 67 s.</x:v>
+      </x:c>
+      <x:c r="I12" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J12" s="13" t="str">
+        <x:v>Reproduzir o exemplo com 82000 Pa e o deslocamento UTC fixo publicado; não substituir pelo fuso civil atual de Denver.</x:v>
+      </x:c>
+      <x:c r="K12" s="13" t="str">
+        <x:v>Date = October 17, 2003</x:v>
+      </x:c>
+      <x:c r="L12" s="13" t="str">
+        <x:v>1b9e2b6131d89ebc17fe4c047e64a0168143c949bfe6fafe06d856d651555cc2</x:v>
+      </x:c>
+      <x:c r="M12" s="13" t="str">
+        <x:v>49d34fdd1e64f32a86006ff36f28eb930ad187a5480273a45b9abed211abeb26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A13" s="13" t="str">
+        <x:v>EV012</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>B32</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>A-16</x:v>
+      </x:c>
+      <x:c r="F13" s="13" t="str">
+        <x:v>A continuação da Tabela A5.1 apresenta zenital e azimute usados na conferência numérica.</x:v>
+      </x:c>
+      <x:c r="G13" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H13" s="13" t="str">
+        <x:v>A Tabela A5.1, p. A-16, imprime zenital 50,11162 e azimute 194,34024 graus. Os resultados calculados coincidem ao arredondar a cinco casas.</x:v>
+      </x:c>
+      <x:c r="I13" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J13" s="13" t="str">
+        <x:v>Usar tolerância de 0,000005 grau, correspondente a meia unidade da última casa impressa; isso verifica implementação e arredondamento, não calibração.</x:v>
+      </x:c>
+      <x:c r="K13" s="13" t="str">
+        <x:v>194.34024</x:v>
+      </x:c>
+      <x:c r="L13" s="13" t="str">
+        <x:v>1b9e2b6131d89ebc17fe4c047e64a0168143c949bfe6fafe06d856d651555cc2</x:v>
+      </x:c>
+      <x:c r="M13" s="13" t="str">
+        <x:v>1d75770e4a205ee905a256a17e73155f84c50c118d15f384216bad2b337b6f7b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A14" s="13" t="str">
+        <x:v>EV013</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>cap. 2-5</x:v>
+      </x:c>
+      <x:c r="F14" s="13" t="str">
+        <x:v>A referência extraterrestre varia com o inverso do quadrado da distância.</x:v>
+      </x:c>
+      <x:c r="G14" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H14" s="13" t="str">
+        <x:v>A equação 2-1 do handbook contém explicitamente o fator (r0/r)^2. O parâmetro solar do projeto é fixado para reprodutibilidade.</x:v>
+      </x:c>
+      <x:c r="I14" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J14" s="13" t="str">
+        <x:v>Manter Gsc=1366,1 W/m2 como parâmetro do software, sem denominá-lo uma determinação metrológica atual da constante solar.</x:v>
+      </x:c>
+      <x:c r="K14" s="13" t="str">
+        <x:v>The Earth’s elliptical orbit</x:v>
+      </x:c>
+      <x:c r="L14" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M14" s="13" t="str">
+        <x:v>73b20a62729471e958bbc8ae4c00bb8590eb081354871b3beb087fb2083f58f5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A15" s="13" t="str">
+        <x:v>EV014</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>cap. 2-8</x:v>
+      </x:c>
+      <x:c r="F15" s="13" t="str">
+        <x:v>A orientação solar local inclui elevação e azimute horário a partir do norte.</x:v>
+      </x:c>
+      <x:c r="G15" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H15" s="13" t="str">
+        <x:v>A seção 2.4.1 confirma elevação e azimute topocêntricos e a convenção norte/leste. A indeterminação no zênite é consequência geométrica da projeção nula.</x:v>
+      </x:c>
+      <x:c r="I15" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J15" s="13" t="str">
+        <x:v>Distinguir definição documentada de consequência matemática; uniformizar A_s nas figuras.</x:v>
+      </x:c>
+      <x:c r="K15" s="13" t="str">
+        <x:v>eastward from true north</x:v>
+      </x:c>
+      <x:c r="L15" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M15" s="13" t="str">
+        <x:v>39e5bde1cd7c142ed75e9f2396975f3385bcd9d5bed66cfc9b81c776054a31cf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="13" t="str">
+        <x:v>EV015</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>B12</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F16" s="13" t="str">
+        <x:v>Irradiação é obtida pela integração temporal da irradiância.</x:v>
+      </x:c>
+      <x:c r="G16" s="13" t="str">
+        <x:v>DIRETA_COM_DERIVACAO</x:v>
+      </x:c>
+      <x:c r="H16" s="13" t="str">
+        <x:v>Duffie define a integral temporal. A soma de médias por duração é derivação matemática sob a hipótese de que o registro representa média do intervalo.</x:v>
+      </x:c>
+      <x:c r="I16" s="13" t="str">
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
+      </x:c>
+      <x:c r="J16" s="13" t="str">
+        <x:v>Identificar E1.04 como forma discreta derivada; somar apenas intervalos válidos e não apresentar energia parcial como energia de toda a janela.</x:v>
+      </x:c>
+      <x:c r="K16" s="13" t="str">
+        <x:v>found by integration of irradiance</x:v>
+      </x:c>
+      <x:c r="L16" s="13" t="str">
+        <x:v>db6ac445398a88a7670cbee02db18c426732e8104ee56e4cfb81fa86be85f4da</x:v>
+      </x:c>
+      <x:c r="M16" s="13" t="str">
+        <x:v>72110de1c76a49763467ae4a724ca8529306562673523078ce77de026ea31f65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A17" s="13" t="str">
+        <x:v>EV016</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>cap. 2-9</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="str">
+        <x:v>DNI, DHI e GHI diferem pelo campo angular e pelo plano de recepção.</x:v>
+      </x:c>
+      <x:c r="G17" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H17" s="13" t="str">
+        <x:v>A seção 2.5 define DNI, DHI e GHI no espectro solar de onda curta e pelos respectivos campos angulares.</x:v>
+      </x:c>
+      <x:c r="I17" s="13" t="str">
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
+      </x:c>
+      <x:c r="J17" s="13" t="str">
+        <x:v>Acrescentar solar/onda curta quando o texto disser irradiância descendente total; distinguir a componente direta ideal da região angular do instrumento.</x:v>
+      </x:c>
+      <x:c r="K17" s="13" t="str">
+        <x:v>three fundamental irradiance components</x:v>
+      </x:c>
+      <x:c r="L17" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M17" s="13" t="str">
+        <x:v>ee304b8b71c286a4f57d4acd8cf30753583cf2ea8f1e337b31a65e52413457bc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A18" s="13" t="str">
+        <x:v>EV017</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>cap. 2-10</x:v>
+      </x:c>
+      <x:c r="F18" s="13" t="str">
+        <x:v>A equação de fechamento soma direta projetada e difusa horizontal.</x:v>
+      </x:c>
+      <x:c r="G18" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H18" s="13" t="str">
+        <x:v>A equação 2-2 contém a soma direta projetada mais difusa. A compatibilidade de banda, plano e suporte temporal é condição de aplicação às medidas.</x:v>
+      </x:c>
+      <x:c r="I18" s="13" t="str">
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
+      </x:c>
+      <x:c r="J18" s="13" t="str">
+        <x:v>Manter fechamento para o Sol acima do horizonte; um resíduo de medidas exige diagnóstico instrumental e temporal, sem atribuição automática.</x:v>
+      </x:c>
+      <x:c r="K18" s="13" t="str">
+        <x:v>fundamental expression called the closure equation</x:v>
+      </x:c>
+      <x:c r="L18" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M18" s="13" t="str">
+        <x:v>2aa583e0de187e08bfda214bed37d731876831601fdf877823b6373708c16437</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A19" s="13" t="str">
+        <x:v>EV018</x:v>
+      </x:c>
+      <x:c r="B19" s="13" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str">
+        <x:v>cap. 2-10</x:v>
+      </x:c>
+      <x:c r="F19" s="13" t="str">
+        <x:v>DNI e DHI estimadas a partir de GHI dependem de modelos de separação.</x:v>
+      </x:c>
+      <x:c r="G19" s="13" t="str">
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
+      </x:c>
+      <x:c r="H19" s="13" t="str">
+        <x:v>A p. 2-10 trata a separação de componentes como modelagem empírica. Driesse et al., pp. 9–11, distinguem o teste de inversão com GTI modelada do confronto com medidas.</x:v>
+      </x:c>
+      <x:c r="I19" s="13" t="str">
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
+      </x:c>
+      <x:c r="J19" s="13" t="str">
+        <x:v>Citar Driesse et al. no limite de identificação: reconvergência ao valor de entrada verifica consistência do procedimento, não valida componentes com observações independentes.</x:v>
+      </x:c>
+      <x:c r="K19" s="13" t="str">
+        <x:v>decomposition</x:v>
+      </x:c>
+      <x:c r="L19" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M19" s="13" t="str">
+        <x:v>2aa583e0de187e08bfda214bed37d731876831601fdf877823b6373708c16437</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A20" s="13" t="str">
+        <x:v>EV019</x:v>
+      </x:c>
+      <x:c r="B20" s="13" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D20" s="13" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E20" s="13" t="str">
+        <x:v>cap. 2-1</x:v>
+      </x:c>
+      <x:c r="F20" s="13" t="str">
+        <x:v>Superfícies fotovoltaicas podem receber contribuições descendentes e refletidas.</x:v>
+      </x:c>
+      <x:c r="G20" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H20" s="13" t="str">
+        <x:v>A introdução do capítulo 2 inclui a contribuição refletida quando está no campo de visão do coletor; a seção 2.5.1 detalha a recepção no plano inclinado.</x:v>
+      </x:c>
+      <x:c r="I20" s="13" t="str">
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
+      </x:c>
+      <x:c r="J20" s="13" t="str">
+        <x:v>Conservar a decomposição conceitual da POA e reservar os modelos de transposição e albedo às seções responsáveis.</x:v>
+      </x:c>
+      <x:c r="K20" s="13" t="str">
+        <x:v>radiation reflected from the ground</x:v>
+      </x:c>
+      <x:c r="L20" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M20" s="13" t="str">
+        <x:v>c4911f6f1f9ad4c7c6c2ee311e21ce59196dbdf1e3474f4495ad274163306439</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A21" s="13" t="str">
+        <x:v>EV020</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E21" s="13" t="str">
+        <x:v>cap. 2-6</x:v>
+      </x:c>
+      <x:c r="F21" s="13" t="str">
+        <x:v>A atmosfera atua sobre a radiação ao longo de um percurso dependente da posição solar.</x:v>
+      </x:c>
+      <x:c r="G21" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H21" s="13" t="str">
+        <x:v>A seção 2.4 relaciona percurso óptico e posição solar; a secante é uma aproximação para zenitais baixos.</x:v>
+      </x:c>
+      <x:c r="I21" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J21" s="13" t="str">
+        <x:v>Vincular ao domínio especificado em Duffie e separar caminho óptico, transmitância e irradiância.</x:v>
+      </x:c>
+      <x:c r="K21" s="13" t="str">
+        <x:v>atmospheric path length or air mass</x:v>
+      </x:c>
+      <x:c r="L21" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M21" s="13" t="str">
+        <x:v>05caf2455788fa82e3522bb49aa84fbc5d484a868d7a17c94b1b008fcbb259a3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A22" s="13" t="str">
+        <x:v>EV021</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="E22" s="13" t="str">
+        <x:v>cap. 2-7</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="str">
+        <x:v>Absorção e espalhamento têm efeitos físicos distintos sobre o campo radiativo.</x:v>
+      </x:c>
+      <x:c r="G22" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H22" s="13" t="str">
+        <x:v>A p. 2-7 distingue captura/absorção e redistribuição angular por espalhamento, inclusive retorno ao espaço.</x:v>
+      </x:c>
+      <x:c r="I22" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J22" s="13" t="str">
+        <x:v>Manter a distinção física; não interpretar espalhamento exclusivamente como energia perdida do sistema terrestre.</x:v>
+      </x:c>
+      <x:c r="K22" s="13" t="str">
+        <x:v>Scattering redistributes the radiation</x:v>
+      </x:c>
+      <x:c r="L22" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M22" s="13" t="str">
+        <x:v>52bb3ce0344ae3d4ac2d3ed00de334fb626de39fa0b94da0ee59ec53d64481ce</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A23" s="13" t="str">
+        <x:v>EV022</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="n">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>cap. 6-2</x:v>
+      </x:c>
+      <x:c r="F23" s="13" t="str">
+        <x:v>Nuvens produzem rampas e podem causar intensificação local de curta duração.</x:v>
+      </x:c>
+      <x:c r="G23" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H23" s="13" t="str">
+        <x:v>A seção 6.2.1 descreve rampas e intensificação local por geometria de nuvens, inclusive valores superiores à referência extraterrestre horizontal.</x:v>
+      </x:c>
+      <x:c r="I23" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J23" s="13" t="str">
+        <x:v>Não usar G0h como teto universal de observações de curta duração nem diagnosticar céu claro pela forma da G01.</x:v>
+      </x:c>
+      <x:c r="K23" s="13" t="str">
+        <x:v>the cloud enhancement phenomenon</x:v>
+      </x:c>
+      <x:c r="L23" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M23" s="13" t="str">
+        <x:v>bb068f26339863b02ff67e175a8c3a99771700b23ec4ef82f5883f0d89e932f8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="50.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>EV023</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="E24" s="13" t="str">
+        <x:v>cap. 5-10</x:v>
+      </x:c>
+      <x:c r="F24" s="13" t="str">
+        <x:v>Aerossóis e vapor de água são descritos por propriedades ópticas e quantidades de coluna.</x:v>
+      </x:c>
+      <x:c r="G24" s="13" t="str">
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
+      </x:c>
+      <x:c r="H24" s="13" t="str">
+        <x:v>A seção 5.6 define AOD espectral e água precipitável integrada na coluna. A não equivalência com umidade relativa superficial decorre de mensurandos e dimensões diferentes.</x:v>
+      </x:c>
+      <x:c r="I24" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J24" s="13" t="str">
+        <x:v>Marcar essa não equivalência como inferência física da definição; não alegar medição de AOD/PW no PVDAQ a partir de POA.</x:v>
+      </x:c>
+      <x:c r="K24" s="13" t="str">
+        <x:v>total column water vapor</x:v>
+      </x:c>
+      <x:c r="L24" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M24" s="13" t="str">
+        <x:v>7b191def666d026d373384de32afd529aadfc9a49bb1dcdbd5bd27c60eac36d2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="13" t="str">
+        <x:v>EV024</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="n">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="E25" s="13" t="str">
+        <x:v>cap. 6-1</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="str">
+        <x:v>A variabilidade deve ser definida em relação ao intervalo temporal e à área.</x:v>
+      </x:c>
+      <x:c r="G25" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H25" s="13" t="str">
+        <x:v>A introdução do capítulo 6 exige definir período e área antes de quantificar variabilidade.</x:v>
+      </x:c>
+      <x:c r="I25" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J25" s="13" t="str">
+        <x:v>Não generalizar o dia mostrado nem o trimestre para distribuição climatológica ou tendência de longo prazo.</x:v>
+      </x:c>
+      <x:c r="K25" s="13" t="str">
+        <x:v>during a specific period</x:v>
+      </x:c>
+      <x:c r="L25" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M25" s="13" t="str">
+        <x:v>64ebe4d4fc87b0918ce49ced541793d90558952c09921b7a675660db2af97b80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A26" s="13" t="str">
+        <x:v>EV025</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C26" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D26" s="13" t="n">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="E26" s="13" t="str">
+        <x:v>cap. 6-2</x:v>
+      </x:c>
+      <x:c r="F26" s="13" t="str">
+        <x:v>A variabilidade depende da componente de irradiância e da escala de análise.</x:v>
+      </x:c>
+      <x:c r="G26" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H26" s="13" t="str">
+        <x:v>A p. 6-2 diferencia variabilidade entre componentes e descreve suavização espacial de rampas em áreas maiores.</x:v>
+      </x:c>
+      <x:c r="I26" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J26" s="13" t="str">
+        <x:v>Informar grandeza e escala; não transferir resultados de DNI instantânea a médias mensais de GHI.</x:v>
+      </x:c>
+      <x:c r="K26" s="13" t="str">
+        <x:v>dependent on the irradiance component</x:v>
+      </x:c>
+      <x:c r="L26" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M26" s="13" t="str">
+        <x:v>bb068f26339863b02ff67e175a8c3a99771700b23ec4ef82f5883f0d89e932f8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="50.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A27" s="13" t="str">
+        <x:v>EV026</x:v>
+      </x:c>
+      <x:c r="B27" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D27" s="13" t="n">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="E27" s="13" t="str">
+        <x:v>cap. 6-17</x:v>
+      </x:c>
+      <x:c r="F27" s="13" t="str">
+        <x:v>Nuvens, relevo e fatores locais limitam extrapolações espaciais do recurso.</x:v>
+      </x:c>
+      <x:c r="G27" s="13" t="str">
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
+      </x:c>
+      <x:c r="H27" s="13" t="str">
+        <x:v>A seção 6.3 documenta heterogeneidade por nuvens, relevo e propriedades atmosféricas. A ausência de garantia de exatidão por pixel menor é inferência sobre os fatores do modelo.</x:v>
+      </x:c>
+      <x:c r="I27" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J27" s="13" t="str">
+        <x:v>Separar resolução nominal de exatidão e exigir comparação local; não apresentar uma relação monotônica universal resolução/erro.</x:v>
+      </x:c>
+      <x:c r="K27" s="13" t="str">
+        <x:v>uncertainty when attempting to extrapolate solar resource data</x:v>
+      </x:c>
+      <x:c r="L27" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M27" s="13" t="str">
+        <x:v>f4deb3f1f66875821a51c4e4f49e867038d39d6bb524362435f8f4321273e94b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A28" s="13" t="str">
+        <x:v>EV027</x:v>
+      </x:c>
+      <x:c r="B28" s="13" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C28" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D28" s="13" t="n">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="E28" s="13" t="str">
+        <x:v>cap. 6-24</x:v>
+      </x:c>
+      <x:c r="F28" s="13" t="str">
+        <x:v>A resolução temporal afeta a variabilidade que pode ser representada na série.</x:v>
+      </x:c>
+      <x:c r="G28" s="13" t="str">
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
+      </x:c>
+      <x:c r="H28" s="13" t="str">
+        <x:v>A seção 6.5 associa variabilidade representada à resolução. A interpolação simples não identifica, por si só, oscilações subintervalo desconhecidas.</x:v>
+      </x:c>
+      <x:c r="I28" s="13" t="str">
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
+      </x:c>
+      <x:c r="J28" s="13" t="str">
+        <x:v>Qualificar a frase sobre interpolação: ela não demonstra recuperação exata da variabilidade ausente sem hipóteses/informação adicionais.</x:v>
+      </x:c>
+      <x:c r="K28" s="13" t="str">
+        <x:v>temporal variability is a direct function</x:v>
+      </x:c>
+      <x:c r="L28" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M28" s="13" t="str">
+        <x:v>0d1cfb9706e46e63228dd11bf1c499bdfac5aede4d1b72c290fe918ff6e6950b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A29" s="13" t="str">
+        <x:v>EV028</x:v>
+      </x:c>
+      <x:c r="B29" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C29" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D29" s="13" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E29" s="13" t="str">
+        <x:v>cap. 3-3</x:v>
+      </x:c>
+      <x:c r="F29" s="13" t="str">
+        <x:v>Medições locais apoiam avaliação do recurso e conferência de modelos.</x:v>
+      </x:c>
+      <x:c r="G29" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H29" s="13" t="str">
+        <x:v>A seção 3.1 apresenta as medições locais como referência para modelos e enumera instalação, operação e manutenção.</x:v>
+      </x:c>
+      <x:c r="I29" s="13" t="str">
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J29" s="13" t="str">
+        <x:v>Manter o papel das observações, sem presumir que todo registro local esteja calibrado ou isento de erros.</x:v>
+      </x:c>
+      <x:c r="K29" s="13" t="str">
+        <x:v>time-consuming and expensive</x:v>
+      </x:c>
+      <x:c r="L29" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M29" s="13" t="str">
+        <x:v>629f6d9ec634c43f965a7a34b01278a6fb00696b5587fe0120eaec4ffe995a28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="50.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A30" s="13" t="str">
+        <x:v>EV029</x:v>
+      </x:c>
+      <x:c r="B30" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C30" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D30" s="13" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E30" s="13" t="str">
+        <x:v>cap. 3-5</x:v>
+      </x:c>
+      <x:c r="F30" s="13" t="str">
+        <x:v>A montagem e o campo de visão distinguem medidas GHI, DHI, DNI e POA.</x:v>
+      </x:c>
+      <x:c r="G30" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H30" s="13" t="str">
+        <x:v>A Tabela 3-1 distingue GHI, DHI, DNI e POA por montagem e campo de visão. Sistemas com sombra rotativa alternam observações e calculam DNI; não são três canais simultâneos independentes.</x:v>
+      </x:c>
+      <x:c r="I30" s="13" t="str">
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J30" s="13" t="str">
+        <x:v>Restringir a afirmação a um sensor em uma montagem fixa; não excluir a existência de sistemas de medição alternada.</x:v>
+      </x:c>
+      <x:c r="K30" s="13" t="str">
+        <x:v>Mounted in the plane of the PV module array</x:v>
+      </x:c>
+      <x:c r="L30" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M30" s="13" t="str">
+        <x:v>ce435002a47688cded151f5f4fd3967faeaf60a0fe4bd7c713a1fb1e91ffdfde</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A31" s="13" t="str">
+        <x:v>EV030</x:v>
+      </x:c>
+      <x:c r="B31" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D31" s="13" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E31" s="13" t="str">
+        <x:v>cap. 3-6</x:v>
+      </x:c>
+      <x:c r="F31" s="13" t="str">
+        <x:v>Termopilhas e sensores fotoelétricos têm respostas espectrais e temporais diferentes.</x:v>
+      </x:c>
+      <x:c r="G31" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H31" s="13" t="str">
+        <x:v>A p. 3-6 contrasta termopilhas e sensores fotoelétricos em resposta temporal e espectral.</x:v>
+      </x:c>
+      <x:c r="I31" s="13" t="str">
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J31" s="13" t="str">
+        <x:v>Distinguir tecnologia de sensor de exatidão de campo; não atribuir ao sensor PVDAQ uma tecnologia não conferida em metadados.</x:v>
+      </x:c>
+      <x:c r="K31" s="13" t="str">
+        <x:v>very fast time-response characteristics</x:v>
+      </x:c>
+      <x:c r="L31" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M31" s="13" t="str">
+        <x:v>f524d6d8266e65bb11d68ec44ce5124b9d2f5106862f27daa203cfe33bcdd1cf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A32" s="13" t="str">
+        <x:v>EV031</x:v>
+      </x:c>
+      <x:c r="B32" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C32" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D32" s="13" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E32" s="13" t="str">
+        <x:v>cap. 3-7</x:v>
+      </x:c>
+      <x:c r="F32" s="13" t="str">
+        <x:v>Pireliômetros requerem alinhamento com o Sol e possuem campo de visão limitado.</x:v>
+      </x:c>
+      <x:c r="G32" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H32" s="13" t="str">
+        <x:v>A seção 3.2.1.1 explicita rastreamento, colimação e contribuição circumsolar no campo de visão finito.</x:v>
+      </x:c>
+      <x:c r="I32" s="13" t="str">
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J32" s="13" t="str">
+        <x:v>Não equiparar sem ressalva DNI instrumental a um feixe matemático de ângulo sólido nulo.</x:v>
+      </x:c>
+      <x:c r="K32" s="13" t="str">
+        <x:v>circumsolar region</x:v>
+      </x:c>
+      <x:c r="L32" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M32" s="13" t="str">
+        <x:v>a155fda84ff8bdd22a9694a7d1c0fde4eea3ac03cf471b4a609b5909e17808f1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A33" s="13" t="str">
+        <x:v>EV032</x:v>
+      </x:c>
+      <x:c r="B33" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D33" s="13" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="E33" s="13" t="str">
+        <x:v>cap. 4-1</x:v>
+      </x:c>
+      <x:c r="F33" s="13" t="str">
+        <x:v>Avaliação e controle de qualidade tratam dados suspeitos e realimentam a operação.</x:v>
+      </x:c>
+      <x:c r="G33" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H33" s="13" t="str">
+        <x:v>O capítulo 4 distingue avaliação posterior dos dados e realimentação do controle operacional.</x:v>
+      </x:c>
+      <x:c r="I33" s="13" t="str">
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J33" s="13" t="str">
+        <x:v>Registrar lacunas e flags; disponibilidade de uma média e completude das amostras são indicadores diferentes.</x:v>
+      </x:c>
+      <x:c r="K33" s="13" t="str">
+        <x:v>flagging suspicious or erroneous data</x:v>
+      </x:c>
+      <x:c r="L33" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M33" s="13" t="str">
+        <x:v>bd54c71cd0de1795065e9fe9d394af882787bf9c606f4813da281725037a041d</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A34" s="13" t="str">
+        <x:v>EV033</x:v>
+      </x:c>
+      <x:c r="B34" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C34" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D34" s="13" t="n">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="E34" s="13" t="str">
+        <x:v>cap. 4-15</x:v>
+      </x:c>
+      <x:c r="F34" s="13" t="str">
+        <x:v>Uma única medição inclinada impõe limitações ao controle de qualidade radiométrico.</x:v>
+      </x:c>
+      <x:c r="G34" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H34" s="13" t="str">
+        <x:v>A p. 4-15 relata dificuldades de QC de GTI/POA de campo, sobretudo com um radiômetro. É uma limitação, não impossibilidade de todo teste.</x:v>
+      </x:c>
+      <x:c r="I34" s="13" t="str">
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J34" s="13" t="str">
+        <x:v>Escrever que a POA isolada restringe testes que exigem componentes independentes; preservar os controles de cadência e disponibilidade que continuam possíveis.</x:v>
+      </x:c>
+      <x:c r="K34" s="13" t="str">
+        <x:v>especially when only a single radiometer exists locally</x:v>
+      </x:c>
+      <x:c r="L34" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M34" s="13" t="str">
+        <x:v>a82a91ce7a98068a76fda15d4a37a4f20ecfc11ae55ee2005b46f04b31f1faa8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A35" s="13" t="str">
+        <x:v>EV034</x:v>
+      </x:c>
+      <x:c r="B35" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C35" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D35" s="13" t="n">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="E35" s="13" t="str">
+        <x:v>cap. 7-1</x:v>
+      </x:c>
+      <x:c r="F35" s="13" t="str">
+        <x:v>Modelos de satélite e adaptação local ampliam a caracterização do recurso.</x:v>
+      </x:c>
+      <x:c r="G35" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H35" s="13" t="str">
+        <x:v>O capítulo 7 resume satélites e adaptação usando observações locais de curto prazo para ajustar séries longas.</x:v>
+      </x:c>
+      <x:c r="I35" s="13" t="str">
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J35" s="13" t="str">
+        <x:v>Não pressupor que essa adaptação foi executada no estudo; descrevê-la como método disponível.</x:v>
+      </x:c>
+      <x:c r="K35" s="13" t="str">
+        <x:v>Site-adaptation models have been used</x:v>
+      </x:c>
+      <x:c r="L35" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M35" s="13" t="str">
+        <x:v>e04bd4129cdb7ea79d3c5754d6a14b1f25d01d39b0631aa03a7327186920bed9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A36" s="13" t="str">
+        <x:v>EV035</x:v>
+      </x:c>
+      <x:c r="B36" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C36" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D36" s="13" t="n">
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="E36" s="13" t="str">
+        <x:v>cap. 7-2</x:v>
+      </x:c>
+      <x:c r="F36" s="13" t="str">
+        <x:v>Reanálises produzem séries históricas de GHI a partir de sistemas atmosféricos.</x:v>
+      </x:c>
+      <x:c r="G36" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H36" s="13" t="str">
+        <x:v>A p. 7-2 identifica ERA5/MERRA-2 como reanálises de modelos atmosféricos. A irradiância superficial é estimada, não uma estação em cada célula.</x:v>
+      </x:c>
+      <x:c r="I36" s="13" t="str">
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J36" s="13" t="str">
+        <x:v>Manter distinção de origem; qualquer resolução ou desempenho numérico requer produto, versão e avaliação próprios.</x:v>
+      </x:c>
+      <x:c r="K36" s="13" t="str">
+        <x:v>reanalysis mode for historical time series</x:v>
+      </x:c>
+      <x:c r="L36" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M36" s="13" t="str">
+        <x:v>5ffab2bcfeb35b43ac12a3b17c20095a55d743516b097980a1b2d10a353ed1a0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A37" s="13" t="str">
+        <x:v>EV036</x:v>
+      </x:c>
+      <x:c r="B37" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C37" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D37" s="13" t="n">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="E37" s="13" t="str">
+        <x:v>cap. 7-8</x:v>
+      </x:c>
+      <x:c r="F37" s="13" t="str">
+        <x:v>Modelos físicos de satélite podem recuperar nuvens e usar transferência radiativa.</x:v>
+      </x:c>
+      <x:c r="G37" s="13" t="str">
+        <x:v>DIRETA</x:v>
+      </x:c>
+      <x:c r="H37" s="13" t="str">
+        <x:v>A p. 7-8 descreve duas etapas: propriedades de nuvens a partir de radiâncias e cálculo superficial por transferência radiativa.</x:v>
+      </x:c>
+      <x:c r="I37" s="13" t="str">
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J37" s="13" t="str">
+        <x:v>Distinguir radiância orbital observada de irradiância superficial estimada.</x:v>
+      </x:c>
+      <x:c r="K37" s="13" t="str">
+        <x:v>derives cloud optical properties</x:v>
+      </x:c>
+      <x:c r="L37" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M37" s="13" t="str">
+        <x:v>2f3e5b467033457d428e47d6249039e158eac4e6cadce7159f513ceee21ab83b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A38" s="13" t="str">
+        <x:v>EV037</x:v>
+      </x:c>
+      <x:c r="B38" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C38" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D38" s="13" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="E38" s="13" t="str">
+        <x:v>cap. 8-4</x:v>
+      </x:c>
+      <x:c r="F38" s="13" t="str">
+        <x:v>Um ano meteorológico típico é uma construção estatística com finalidade própria.</x:v>
+      </x:c>
+      <x:c r="G38" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H38" s="13" t="str">
+        <x:v>A p. 8-4 descreve concatenação de meses típicos e exclui o uso para um período histórico específico ou condições extremas de projeto.</x:v>
+      </x:c>
+      <x:c r="I38" s="13" t="str">
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J38" s="13" t="str">
+        <x:v>Não chamar TMY de ano observado integral nem usá-lo para reconstituir abril–junho de 2024.</x:v>
+      </x:c>
+      <x:c r="K38" s="13" t="str">
+        <x:v>TMY data are not designed to provide meteorological extremes</x:v>
+      </x:c>
+      <x:c r="L38" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M38" s="13" t="str">
+        <x:v>112212d8bbb75d4c1edd9120b2dee8ca38d3800b51a5068ae603720f1ed83043</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A39" s="13" t="str">
+        <x:v>EV038</x:v>
+      </x:c>
+      <x:c r="B39" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C39" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D39" s="13" t="n">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="E39" s="13" t="str">
+        <x:v>cap. 10-5</x:v>
+      </x:c>
+      <x:c r="F39" s="13" t="str">
+        <x:v>Incerteza depende do mensurando e de contribuições da medição e da calibração.</x:v>
+      </x:c>
+      <x:c r="G39" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H39" s="13" t="str">
+        <x:v>A seção 10.2 exige mensurando, unidade e incerteza, enumerando contribuições de instrumento, aquisição, ambiente e calibração.</x:v>
+      </x:c>
+      <x:c r="I39" s="13" t="str">
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J39" s="13" t="str">
+        <x:v>Não usar completude, correlação ou uma métrica de erro como estimativa completa da incerteza; nenhuma incerteza do sensor foi calculada nesta seção.</x:v>
+      </x:c>
+      <x:c r="K39" s="13" t="str">
+        <x:v>the measurand has four general sources of uncertainty</x:v>
+      </x:c>
+      <x:c r="L39" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M39" s="13" t="str">
+        <x:v>aaa43c4da0d962ac7a41e9b7fe4f52555fd63584a7b6d21f1d7e1cd9af5bd44a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="33.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A40" s="13" t="str">
+        <x:v>EV039</x:v>
+      </x:c>
+      <x:c r="B40" s="13" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C40" s="13" t="str">
+        <x:v>A045</x:v>
+      </x:c>
+      <x:c r="D40" s="13" t="n">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="E40" s="13" t="str">
+        <x:v>cap. 10-6</x:v>
+      </x:c>
+      <x:c r="F40" s="13" t="str">
+        <x:v>Modelos, entradas, propagação e referência contribuem para a incerteza estimada.</x:v>
+      </x:c>
+      <x:c r="G40" s="13" t="str">
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
+      </x:c>
+      <x:c r="H40" s="13" t="str">
+        <x:v>A p. 10-6 enumera modelo, entradas, propagação, referência, variabilidade interanual e tendências. A quantificação depende de lugar e período.</x:v>
+      </x:c>
+      <x:c r="I40" s="13" t="str">
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
+      </x:c>
+      <x:c r="J40" s="13" t="str">
+        <x:v>Manter discussão conceitual e encaminhar a quantificação de desempenho à Seção 4, sem criar valores de incerteza não executados.</x:v>
+      </x:c>
+      <x:c r="K40" s="13" t="str">
+        <x:v>uncertainty in its input data</x:v>
+      </x:c>
+      <x:c r="L40" s="13" t="str">
+        <x:v>cfe5e510b7a2a05a18e8660af346454a5e7c9a704b5b5a02533a67e04a2de26a</x:v>
+      </x:c>
+      <x:c r="M40" s="13" t="str">
+        <x:v>6e1ad0e2406810718ba03206450ad0ac19dcd293dc963a30ff497ff77058c32d</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9adf9eba4924bd7"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -655,13 +2344,13 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
       <x:c r="L3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O3" s="6" t="str">
         <x:v>Não substituir silenciosamente por A003.</x:v>
@@ -745,13 +2434,13 @@
       </x:c>
       <x:c r="K5" s="6" t="str"/>
       <x:c r="L5" s="6" t="str">
-        <x:v>Documentação e código conferidos</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M5" s="6" t="str">
-        <x:v>Versão e uso registrados; não é leitura de PDF</x:v>
+        <x:v>prioritária; leitura localizada</x:v>
       </x:c>
       <x:c r="N5" s="6" t="str">
-        <x:v>prioritária; leitura localizada</x:v>
+        <x:v>fundamento de afirmações verificadas</x:v>
       </x:c>
       <x:c r="O5" s="6" t="str">
         <x:v>Cálculo da irradiância extraterrestre normal.</x:v>
@@ -957,13 +2646,13 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
       <x:c r="L2" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>1,9,10,11</x:v>
       </x:c>
       <x:c r="M2" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>complementar selecionada; pp. 1 e 9–11 conferidas; limites da validação inversa</x:v>
       </x:c>
       <x:c r="N2" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>fundamento de afirmações verificadas</x:v>
       </x:c>
       <x:c r="O2" s="6" t="str">
         <x:v>Modelo de céu e componentes para transposição.</x:v>
@@ -1047,13 +2736,13 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
       <x:c r="L4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="N4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O4" s="6" t="str">
         <x:v>Não substituir silenciosamente por A003.</x:v>
@@ -1090,13 +2779,13 @@
       </x:c>
       <x:c r="K5" s="6" t="str"/>
       <x:c r="L5" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M5" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="N5" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O5" s="6" t="str">
         <x:v>A034 é a 1ª edição de 2003, apenas apoio.</x:v>
@@ -1133,13 +2822,13 @@
       </x:c>
       <x:c r="K6" s="6" t="str"/>
       <x:c r="L6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>dados preparados conferidos; citação DOI confirmada em material DOE/NREL, p. 25</x:v>
       </x:c>
       <x:c r="N6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O6" s="6" t="str">
         <x:v>Dados de campo POA/geração; sem GHI/DNI/DHI locais medidos.</x:v>
@@ -1178,13 +2867,13 @@
       </x:c>
       <x:c r="K7" s="6" t="str"/>
       <x:c r="L7" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>26,28,29,55</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova; PDF disponível com fontes e recursos gráficos danificados; 4ª edição lida separadamente</x:v>
       </x:c>
       <x:c r="N7" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O7" s="6" t="str">
         <x:v>PDF consultado é o formato IEA PVPS; DOI aponta para o formato NREL.</x:v>
@@ -1341,13 +3030,13 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
       <x:c r="L3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O3" s="6" t="str">
         <x:v>Não substituir silenciosamente por A003.</x:v>
@@ -1384,13 +3073,13 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
       <x:c r="L4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>dados preparados conferidos; citação DOI confirmada em material DOE/NREL, p. 25</x:v>
       </x:c>
       <x:c r="N4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O4" s="6" t="str">
         <x:v>Dados de campo POA/geração; sem GHI/DNI/DHI locais medidos.</x:v>
@@ -1427,13 +3116,13 @@
       </x:c>
       <x:c r="K5" s="6" t="str"/>
       <x:c r="L5" s="6" t="str">
-        <x:v>Contexto online conferido</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M5" s="6" t="str">
-        <x:v>Versão e uso registrados; não é leitura de PDF</x:v>
+        <x:v>contexto online conferido; fora da fundamentação principal</x:v>
       </x:c>
       <x:c r="N5" s="6" t="str">
-        <x:v>contexto online conferido; fora da fundamentação principal</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O5" s="6" t="str">
         <x:v>Contextualização do Farm Solar Array e do tratamento de dados.</x:v>
@@ -1472,13 +3161,13 @@
       </x:c>
       <x:c r="K6" s="6" t="str"/>
       <x:c r="L6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>26,28,29,55</x:v>
       </x:c>
       <x:c r="M6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova; PDF disponível com fontes e recursos gráficos danificados; 4ª edição lida separadamente</x:v>
       </x:c>
       <x:c r="N6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O6" s="6" t="str">
         <x:v>PDF consultado é o formato IEA PVPS; DOI aponta para o formato NREL.</x:v>
@@ -1635,13 +3324,13 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
       <x:c r="L3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O3" s="6" t="str">
         <x:v>Não substituir silenciosamente por A003.</x:v>
@@ -1678,13 +3367,13 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
       <x:c r="L4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>dados preparados conferidos; citação DOI confirmada em material DOE/NREL, p. 25</x:v>
       </x:c>
       <x:c r="N4" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O4" s="6" t="str">
         <x:v>Dados de campo POA/geração; sem GHI/DNI/DHI locais medidos.</x:v>
@@ -1721,13 +3410,13 @@
       </x:c>
       <x:c r="K5" s="6" t="str"/>
       <x:c r="L5" s="6" t="str">
-        <x:v>Contexto online conferido</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M5" s="6" t="str">
-        <x:v>Versão e uso registrados; não é leitura de PDF</x:v>
+        <x:v>contexto online conferido; fora da fundamentação principal</x:v>
       </x:c>
       <x:c r="N5" s="6" t="str">
-        <x:v>contexto online conferido; fora da fundamentação principal</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O5" s="6" t="str">
         <x:v>Contextualização do Farm Solar Array e do tratamento de dados.</x:v>
@@ -1764,13 +3453,13 @@
       </x:c>
       <x:c r="K6" s="6" t="str"/>
       <x:c r="L6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Decisão documentada</x:v>
       </x:c>
       <x:c r="M6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>README oficial conferido; proveniência e acesso; sem presumir leitura de todo o acervo</x:v>
       </x:c>
       <x:c r="N6" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O6" s="6" t="str">
         <x:v>Acesso e proveniência técnica do conjunto de dados.</x:v>
@@ -1809,13 +3498,13 @@
       </x:c>
       <x:c r="K7" s="6" t="str"/>
       <x:c r="L7" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>26,28,29,55</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>não selecionada como prova; PDF disponível com fontes e recursos gráficos danificados; 4ª edição lida separadamente</x:v>
       </x:c>
       <x:c r="N7" s="6" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="O7" s="6" t="str">
         <x:v>PDF consultado é o formato IEA PVPS; DOI aponta para o formato NREL.</x:v>
@@ -2898,7 +4587,7 @@
         <x:v>Leitura integral</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="2" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -2914,7 +4603,9 @@
       <x:c r="E2" s="13" t="str">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="F2" s="13" t="str"/>
+      <x:c r="F2" s="13" t="str">
+        <x:v>Variation of the earth-sun distance</x:v>
+      </x:c>
       <x:c r="G2" s="13" t="str">
         <x:v>A distância Terra–Sol modifica a irradiância extraterrestre normal.</x:v>
       </x:c>
@@ -2934,10 +4625,10 @@
         <x:v>Leitura localizada; coeficiente de Spencer cotejado com o código.</x:v>
       </x:c>
       <x:c r="M2" s="13" t="str">
-        <x:v>Spencer cotejado com pvlib 0.16.1</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N2" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O2" s="13" t="str">
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
@@ -2958,7 +4649,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="16.799999237060547" hidden="0" customHeight="1">
+    <x:row r="3" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A3" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -2974,7 +4665,9 @@
       <x:c r="E3" s="13" t="str">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F3" s="13" t="str"/>
+      <x:c r="F3" s="13" t="str">
+        <x:v>the angle between the vertical and the line to the sun</x:v>
+      </x:c>
       <x:c r="G3" s="13" t="str">
         <x:v>Zenital é contado desde a vertical; elevação é seu complemento.</x:v>
       </x:c>
@@ -2994,10 +4687,10 @@
         <x:v>Esquema geométrico; sem refração.</x:v>
       </x:c>
       <x:c r="M3" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N3" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O3" s="13" t="str">
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
@@ -3018,7 +4711,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="16.799999237060547" hidden="0" customHeight="1">
+    <x:row r="4" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A4" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3034,7 +4727,9 @@
       <x:c r="E4" s="13" t="str">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F4" s="13" t="str"/>
+      <x:c r="F4" s="13" t="str">
+        <x:v>the angle of incidence is the zenith angle</x:v>
+      </x:c>
       <x:c r="G4" s="13" t="str">
         <x:v>A relação esférica liga latitude, declinação e ângulo horário ao zenital.</x:v>
       </x:c>
@@ -3054,10 +4749,10 @@
         <x:v>A equação elementar não substitui todos os termos do SPA.</x:v>
       </x:c>
       <x:c r="M4" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N4" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O4" s="13" t="str">
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
@@ -3078,7 +4773,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="5" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A5" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3094,7 +4789,9 @@
       <x:c r="E5" s="13" t="str">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="str"/>
+      <x:c r="F5" s="13" t="str">
+        <x:v>east of south are negative</x:v>
+      </x:c>
       <x:c r="G5" s="13" t="str">
         <x:v>O livro adota origem azimutal no sul, com sinais distintos da convenção SPA.</x:v>
       </x:c>
@@ -3114,10 +4811,10 @@
         <x:v>Conversão de origem explicitada; não transcrever convenções como equivalentes.</x:v>
       </x:c>
       <x:c r="M5" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N5" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O5" s="13" t="str">
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
@@ -3138,7 +4835,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="6" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A6" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3154,9 +4851,11 @@
       <x:c r="E6" s="13" t="str">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="F6" s="13" t="str"/>
+      <x:c r="F6" s="13" t="str">
+        <x:v>at sea level</x:v>
+      </x:c>
       <x:c r="G6" s="13" t="str">
-        <x:v>A aproximação secante da massa de ar é apresentada para zenitais até cerca de 70°.</x:v>
+        <x:v>Ao nível do mar, a aproximação secante da massa de ar é apresentada para zenitais até cerca de 70°.</x:v>
       </x:c>
       <x:c r="H6" s="13" t="str">
         <x:v>Massa de ar</x:v>
@@ -3171,13 +4870,13 @@
         <x:v>1.1.4</x:v>
       </x:c>
       <x:c r="L6" s="13" t="str">
-        <x:v>Não extrapolar ao horizonte.</x:v>
+        <x:v>Domínio de atmosfera plana; não extrapolar ao horizonte.</x:v>
       </x:c>
       <x:c r="M6" s="13" t="str">
-        <x:v>Spencer cotejado com pvlib 0.16.1</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N6" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O6" s="13" t="str">
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
@@ -3198,7 +4897,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="7" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A7" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3214,7 +4913,9 @@
       <x:c r="E7" s="13" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="13" t="str"/>
+      <x:c r="F7" s="13" t="str">
+        <x:v>the true solar time</x:v>
+      </x:c>
       <x:c r="G7" s="13" t="str">
         <x:v>O tempo solar verdadeiro depende de longitude, fuso e equação do tempo.</x:v>
       </x:c>
@@ -3234,10 +4935,10 @@
         <x:v>Algoritmo aproximado; não é a implementação SPA utilizada.</x:v>
       </x:c>
       <x:c r="M7" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N7" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O7" s="13" t="str">
         <x:v>https://gml.noaa.gov/grad/solcalc/solareqns.PDF</x:v>
@@ -3258,7 +4959,7 @@
         <x:v>Sim</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="8" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A8" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3274,9 +4975,11 @@
       <x:c r="E8" s="13" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F8" s="13" t="str"/>
+      <x:c r="F8" s="13" t="str">
+        <x:v>size of the solar disk</x:v>
+      </x:c>
       <x:c r="G8" s="13" t="str">
-        <x:v>A formulação de nascer e pôr do Sol acrescenta uma correção aproximada ao horizonte.</x:v>
+        <x:v>O critério de nascer e pôr do Sol em 90,833° inclui aproximações de refração e tamanho angular do disco solar.</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
         <x:v>Horizonte</x:v>
@@ -3294,10 +4997,10 @@
         <x:v>Critério de horizonte aparente difere do recorte geométrico de G0h.</x:v>
       </x:c>
       <x:c r="M8" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N8" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O8" s="13" t="str">
         <x:v>https://gml.noaa.gov/grad/solcalc/solareqns.PDF</x:v>
@@ -3318,7 +5021,7 @@
         <x:v>Sim</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="9" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3334,7 +5037,9 @@
       <x:c r="E9" s="13" t="str">
         <x:v>577</x:v>
       </x:c>
-      <x:c r="F9" s="13" t="str"/>
+      <x:c r="F9" s="13" t="str">
+        <x:v>measured from north and eastward</x:v>
+      </x:c>
       <x:c r="G9" s="13" t="str">
         <x:v>O artigo SPA explicita azimute desde o norte e longitude positiva para leste.</x:v>
       </x:c>
@@ -3354,10 +5059,10 @@
         <x:v>Convenção utilizada no capítulo.</x:v>
       </x:c>
       <x:c r="M9" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N9" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O9" s="13" t="str">
         <x:v>https://doi.org/10.1016/j.solener.2003.12.003</x:v>
@@ -3378,7 +5083,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="10" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A10" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3394,7 +5099,9 @@
       <x:c r="E10" s="13" t="str">
         <x:v>578</x:v>
       </x:c>
-      <x:c r="F10" s="13" t="str"/>
+      <x:c r="F10" s="13" t="str">
+        <x:v>In this report we describe a procedure</x:v>
+      </x:c>
       <x:c r="G10" s="13" t="str">
         <x:v>A precisão angular atribuída ao SPA se refere ao cálculo de posição solar.</x:v>
       </x:c>
@@ -3414,10 +5121,10 @@
         <x:v>Não representa a incerteza de um sensor de irradiância.</x:v>
       </x:c>
       <x:c r="M10" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N10" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O10" s="13" t="str">
         <x:v>https://doi.org/10.1016/j.solener.2003.12.003</x:v>
@@ -3438,7 +5145,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="11" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A11" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3454,7 +5161,9 @@
       <x:c r="E11" s="13" t="str">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F11" s="13" t="str"/>
+      <x:c r="F11" s="13" t="str">
+        <x:v>without atmospheric refraction correction</x:v>
+      </x:c>
       <x:c r="G11" s="13" t="str">
         <x:v>O tratamento topocêntrico distingue elevação sem e com refração.</x:v>
       </x:c>
@@ -3474,10 +5183,10 @@
         <x:v>Refração depende de pressão e temperatura; continuação na p. 11/PDF17.</x:v>
       </x:c>
       <x:c r="M11" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N11" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O11" s="13" t="str">
         <x:v>https://doi.org/10.2172/15003974</x:v>
@@ -3498,7 +5207,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="12" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A12" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3514,7 +5223,9 @@
       <x:c r="E12" s="13" t="str">
         <x:v>A-15</x:v>
       </x:c>
-      <x:c r="F12" s="13" t="str"/>
+      <x:c r="F12" s="13" t="str">
+        <x:v>Date = October 17, 2003</x:v>
+      </x:c>
       <x:c r="G12" s="13" t="str">
         <x:v>O exemplo numérico informa data, fuso, localização, pressão, altitude, temperatura e ΔT.</x:v>
       </x:c>
@@ -3534,10 +5245,10 @@
         <x:v>Exemplo de implementação; não é observação PVDAQ.</x:v>
       </x:c>
       <x:c r="M12" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N12" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O12" s="13" t="str">
         <x:v>https://doi.org/10.2172/15003974</x:v>
@@ -3558,7 +5269,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="13" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A13" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3574,7 +5285,9 @@
       <x:c r="E13" s="13" t="str">
         <x:v>A-16</x:v>
       </x:c>
-      <x:c r="F13" s="13" t="str"/>
+      <x:c r="F13" s="13" t="str">
+        <x:v>194.34024</x:v>
+      </x:c>
       <x:c r="G13" s="13" t="str">
         <x:v>A continuação da Tabela A5.1 apresenta zenital e azimute usados na conferência numérica.</x:v>
       </x:c>
@@ -3594,10 +5307,10 @@
         <x:v>Comparação com os valores arredondados da tabela.</x:v>
       </x:c>
       <x:c r="M13" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N13" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O13" s="13" t="str">
         <x:v>https://doi.org/10.2172/15003974</x:v>
@@ -3618,7 +5331,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="14" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A14" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3634,7 +5347,9 @@
       <x:c r="E14" s="13" t="str">
         <x:v>cap. 2-5</x:v>
       </x:c>
-      <x:c r="F14" s="13" t="str"/>
+      <x:c r="F14" s="13" t="str">
+        <x:v>The Earth’s elliptical orbit</x:v>
+      </x:c>
       <x:c r="G14" s="13" t="str">
         <x:v>A referência extraterrestre varia com o inverso do quadrado da distância.</x:v>
       </x:c>
@@ -3654,10 +5369,10 @@
         <x:v>Não equivale à irradiância de superfície.</x:v>
       </x:c>
       <x:c r="M14" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N14" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O14" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -3678,7 +5393,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="15" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A15" s="13" t="str">
         <x:v>1.1</x:v>
       </x:c>
@@ -3694,7 +5409,9 @@
       <x:c r="E15" s="13" t="str">
         <x:v>cap. 2-8</x:v>
       </x:c>
-      <x:c r="F15" s="13" t="str"/>
+      <x:c r="F15" s="13" t="str">
+        <x:v>eastward from true north</x:v>
+      </x:c>
       <x:c r="G15" s="13" t="str">
         <x:v>A orientação solar local inclui elevação e azimute horário a partir do norte.</x:v>
       </x:c>
@@ -3714,10 +5431,10 @@
         <x:v>Azimute indefinido no zênite é uma consequência geométrica.</x:v>
       </x:c>
       <x:c r="M15" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N15" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O15" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -3738,7 +5455,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="16.799999237060547" hidden="0" customHeight="1">
+    <x:row r="16" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A16" s="13" t="str">
         <x:v>1.2</x:v>
       </x:c>
@@ -3754,7 +5471,9 @@
       <x:c r="E16" s="13" t="str">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F16" s="13" t="str"/>
+      <x:c r="F16" s="13" t="str">
+        <x:v>found by integration of irradiance</x:v>
+      </x:c>
       <x:c r="G16" s="13" t="str">
         <x:v>Irradiação é obtida pela integração temporal da irradiância.</x:v>
       </x:c>
@@ -3774,10 +5493,10 @@
         <x:v>A soma utiliza a duração e o significado dos registros.</x:v>
       </x:c>
       <x:c r="M16" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie pp. 9–15, NOAA p. 1–2 e SPA pp. 10–11: comparar fórmulas, convenções e hipóteses; não são medições PVDAQ.</x:v>
       </x:c>
       <x:c r="N16" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_DERIVACAO</x:v>
       </x:c>
       <x:c r="O16" s="13" t="str">
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
@@ -3798,7 +5517,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="17" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A17" s="13" t="str">
         <x:v>1.2</x:v>
       </x:c>
@@ -3814,7 +5533,9 @@
       <x:c r="E17" s="13" t="str">
         <x:v>cap. 2-9</x:v>
       </x:c>
-      <x:c r="F17" s="13" t="str"/>
+      <x:c r="F17" s="13" t="str">
+        <x:v>three fundamental irradiance components</x:v>
+      </x:c>
       <x:c r="G17" s="13" t="str">
         <x:v>DNI, DHI e GHI diferem pelo campo angular e pelo plano de recepção.</x:v>
       </x:c>
@@ -3831,13 +5552,13 @@
         <x:v>1.2.2</x:v>
       </x:c>
       <x:c r="L17" s="13" t="str">
-        <x:v>Grandezas do campo radiativo descendente.</x:v>
+        <x:v>Grandezas do campo solar descendente de ondas curtas.</x:v>
       </x:c>
       <x:c r="M17" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
       </x:c>
       <x:c r="N17" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O17" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -3858,7 +5579,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="18" ht="84" hidden="0" customHeight="1">
       <x:c r="A18" s="13" t="str">
         <x:v>1.2</x:v>
       </x:c>
@@ -3874,7 +5595,9 @@
       <x:c r="E18" s="13" t="str">
         <x:v>cap. 2-10</x:v>
       </x:c>
-      <x:c r="F18" s="13" t="str"/>
+      <x:c r="F18" s="13" t="str">
+        <x:v>fundamental expression called the closure equation</x:v>
+      </x:c>
       <x:c r="G18" s="13" t="str">
         <x:v>A equação de fechamento soma direta projetada e difusa horizontal.</x:v>
       </x:c>
@@ -3894,10 +5617,10 @@
         <x:v>Medições precisam ser compatíveis em banda, campo angular e tempo.</x:v>
       </x:c>
       <x:c r="M18" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
       </x:c>
       <x:c r="N18" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O18" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -3918,7 +5641,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="19" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A19" s="13" t="str">
         <x:v>1.2</x:v>
       </x:c>
@@ -3934,7 +5657,9 @@
       <x:c r="E19" s="13" t="str">
         <x:v>cap. 2-10</x:v>
       </x:c>
-      <x:c r="F19" s="13" t="str"/>
+      <x:c r="F19" s="13" t="str">
+        <x:v>decomposition</x:v>
+      </x:c>
       <x:c r="G19" s="13" t="str">
         <x:v>DNI e DHI estimadas a partir de GHI dependem de modelos de separação.</x:v>
       </x:c>
@@ -3954,10 +5679,10 @@
         <x:v>Não constituem medições adicionais independentes.</x:v>
       </x:c>
       <x:c r="M19" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
       </x:c>
       <x:c r="N19" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
       </x:c>
       <x:c r="O19" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -3978,7 +5703,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="20" ht="50.400001525878906" hidden="0" customHeight="1">
       <x:c r="A20" s="13" t="str">
         <x:v>1.2</x:v>
       </x:c>
@@ -3994,7 +5719,9 @@
       <x:c r="E20" s="13" t="str">
         <x:v>cap. 2-1</x:v>
       </x:c>
-      <x:c r="F20" s="13" t="str"/>
+      <x:c r="F20" s="13" t="str">
+        <x:v>radiation reflected from the ground</x:v>
+      </x:c>
       <x:c r="G20" s="13" t="str">
         <x:v>Superfícies fotovoltaicas podem receber contribuições descendentes e refletidas.</x:v>
       </x:c>
@@ -4014,10 +5741,10 @@
         <x:v>Modelos de transposição pertencem à subseção 3.1.</x:v>
       </x:c>
       <x:c r="M20" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Duffie p. 10; handbook cap. 2-9–2-11; Driesse et al. pp. 9–11 para o limite de validação da inversão.</x:v>
       </x:c>
       <x:c r="N20" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O20" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4038,7 +5765,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="21" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A21" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4054,7 +5781,9 @@
       <x:c r="E21" s="13" t="str">
         <x:v>cap. 2-6</x:v>
       </x:c>
-      <x:c r="F21" s="13" t="str"/>
+      <x:c r="F21" s="13" t="str">
+        <x:v>atmospheric path length or air mass</x:v>
+      </x:c>
       <x:c r="G21" s="13" t="str">
         <x:v>A atmosfera atua sobre a radiação ao longo de um percurso dependente da posição solar.</x:v>
       </x:c>
@@ -4074,10 +5803,10 @@
         <x:v>A secante é uma aproximação limitada.</x:v>
       </x:c>
       <x:c r="M21" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N21" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O21" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4098,7 +5827,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="22" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A22" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4114,7 +5843,9 @@
       <x:c r="E22" s="13" t="str">
         <x:v>cap. 2-7</x:v>
       </x:c>
-      <x:c r="F22" s="13" t="str"/>
+      <x:c r="F22" s="13" t="str">
+        <x:v>Scattering redistributes the radiation</x:v>
+      </x:c>
       <x:c r="G22" s="13" t="str">
         <x:v>Absorção e espalhamento têm efeitos físicos distintos sobre o campo radiativo.</x:v>
       </x:c>
@@ -4134,10 +5865,10 @@
         <x:v>Redistribuição angular não equivale à absorção.</x:v>
       </x:c>
       <x:c r="M22" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N22" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O22" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4158,7 +5889,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="23" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A23" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4174,7 +5905,9 @@
       <x:c r="E23" s="13" t="str">
         <x:v>cap. 6-2</x:v>
       </x:c>
-      <x:c r="F23" s="13" t="str"/>
+      <x:c r="F23" s="13" t="str">
+        <x:v>the cloud enhancement phenomenon</x:v>
+      </x:c>
       <x:c r="G23" s="13" t="str">
         <x:v>Nuvens produzem rampas e podem causar intensificação local de curta duração.</x:v>
       </x:c>
@@ -4194,10 +5927,10 @@
         <x:v>Não classificar céu claro apenas pela forma de POA.</x:v>
       </x:c>
       <x:c r="M23" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N23" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O23" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4218,7 +5951,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="24" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A24" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4234,7 +5967,9 @@
       <x:c r="E24" s="13" t="str">
         <x:v>cap. 5-10</x:v>
       </x:c>
-      <x:c r="F24" s="13" t="str"/>
+      <x:c r="F24" s="13" t="str">
+        <x:v>total column water vapor</x:v>
+      </x:c>
       <x:c r="G24" s="13" t="str">
         <x:v>Aerossóis e vapor de água são descritos por propriedades ópticas e quantidades de coluna.</x:v>
       </x:c>
@@ -4254,10 +5989,10 @@
         <x:v>Umidade relativa superficial não substitui água precipitável.</x:v>
       </x:c>
       <x:c r="M24" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N24" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
       </x:c>
       <x:c r="O24" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4278,7 +6013,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="25" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A25" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4294,7 +6029,9 @@
       <x:c r="E25" s="13" t="str">
         <x:v>cap. 6-1</x:v>
       </x:c>
-      <x:c r="F25" s="13" t="str"/>
+      <x:c r="F25" s="13" t="str">
+        <x:v>during a specific period</x:v>
+      </x:c>
       <x:c r="G25" s="13" t="str">
         <x:v>A variabilidade deve ser definida em relação ao intervalo temporal e à área.</x:v>
       </x:c>
@@ -4314,10 +6051,10 @@
         <x:v>Não generalizar um dia para climatologia.</x:v>
       </x:c>
       <x:c r="M25" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N25" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O25" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4338,7 +6075,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="26" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A26" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4354,7 +6091,9 @@
       <x:c r="E26" s="13" t="str">
         <x:v>cap. 6-2</x:v>
       </x:c>
-      <x:c r="F26" s="13" t="str"/>
+      <x:c r="F26" s="13" t="str">
+        <x:v>dependent on the irradiance component</x:v>
+      </x:c>
       <x:c r="G26" s="13" t="str">
         <x:v>A variabilidade depende da componente de irradiância e da escala de análise.</x:v>
       </x:c>
@@ -4374,10 +6113,10 @@
         <x:v>Agregação espacial pode suavizar oscilações rápidas.</x:v>
       </x:c>
       <x:c r="M26" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N26" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O26" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4398,7 +6137,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="27" ht="100.80000305175781" hidden="0" customHeight="1">
       <x:c r="A27" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4414,7 +6153,9 @@
       <x:c r="E27" s="13" t="str">
         <x:v>cap. 6-17</x:v>
       </x:c>
-      <x:c r="F27" s="13" t="str"/>
+      <x:c r="F27" s="13" t="str">
+        <x:v>uncertainty when attempting to extrapolate solar resource data</x:v>
+      </x:c>
       <x:c r="G27" s="13" t="str">
         <x:v>Nuvens, relevo e fatores locais limitam extrapolações espaciais do recurso.</x:v>
       </x:c>
@@ -4434,10 +6175,10 @@
         <x:v>Pixel menor não garante, sozinho, maior exatidão.</x:v>
       </x:c>
       <x:c r="M27" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N27" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
       </x:c>
       <x:c r="O27" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4458,7 +6199,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="28" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A28" s="13" t="str">
         <x:v>1.3</x:v>
       </x:c>
@@ -4474,7 +6215,9 @@
       <x:c r="E28" s="13" t="str">
         <x:v>cap. 6-24</x:v>
       </x:c>
-      <x:c r="F28" s="13" t="str"/>
+      <x:c r="F28" s="13" t="str">
+        <x:v>temporal variability is a direct function</x:v>
+      </x:c>
       <x:c r="G28" s="13" t="str">
         <x:v>A resolução temporal afeta a variabilidade que pode ser representada na série.</x:v>
       </x:c>
@@ -4491,13 +6234,13 @@
         <x:v>1.3.2; 1.4.3</x:v>
       </x:c>
       <x:c r="L28" s="13" t="str">
-        <x:v>Interpolação não recupera variabilidade não observada.</x:v>
+        <x:v>Interpolação, por si só, não demonstra recuperação exata de oscilações desconhecidas sem hipóteses adicionais.</x:v>
       </x:c>
       <x:c r="M28" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições do cap. 2, propriedades do cap. 5 e escalas do cap. 6 do mesmo handbook; não contabilizar como estudos independentes.</x:v>
       </x:c>
       <x:c r="N28" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_INFERENCIA</x:v>
       </x:c>
       <x:c r="O28" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4518,7 +6261,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="29" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A29" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4534,7 +6277,9 @@
       <x:c r="E29" s="13" t="str">
         <x:v>cap. 3-3</x:v>
       </x:c>
-      <x:c r="F29" s="13" t="str"/>
+      <x:c r="F29" s="13" t="str">
+        <x:v>time-consuming and expensive</x:v>
+      </x:c>
       <x:c r="G29" s="13" t="str">
         <x:v>Medições locais apoiam avaliação do recurso e conferência de modelos.</x:v>
       </x:c>
@@ -4554,10 +6299,10 @@
         <x:v>Existem custos de instalação, operação e manutenção.</x:v>
       </x:c>
       <x:c r="M29" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N29" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O29" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4578,7 +6323,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="30" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A30" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4594,7 +6339,9 @@
       <x:c r="E30" s="13" t="str">
         <x:v>cap. 3-5</x:v>
       </x:c>
-      <x:c r="F30" s="13" t="str"/>
+      <x:c r="F30" s="13" t="str">
+        <x:v>Mounted in the plane of the PV module array</x:v>
+      </x:c>
       <x:c r="G30" s="13" t="str">
         <x:v>A montagem e o campo de visão distinguem medidas GHI, DHI, DNI e POA.</x:v>
       </x:c>
@@ -4611,13 +6358,13 @@
         <x:v>1.4.1</x:v>
       </x:c>
       <x:c r="L30" s="13" t="str">
-        <x:v>Um sensor não mede todas as componentes simultaneamente.</x:v>
+        <x:v>Uma montagem fixa não fornece todos os canais independentes; sistemas de sombra rotativa alternam medições e calculam DNI.</x:v>
       </x:c>
       <x:c r="M30" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N30" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O30" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4638,7 +6385,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="31" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A31" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4654,7 +6401,9 @@
       <x:c r="E31" s="13" t="str">
         <x:v>cap. 3-6</x:v>
       </x:c>
-      <x:c r="F31" s="13" t="str"/>
+      <x:c r="F31" s="13" t="str">
+        <x:v>very fast time-response characteristics</x:v>
+      </x:c>
       <x:c r="G31" s="13" t="str">
         <x:v>Termopilhas e sensores fotoelétricos têm respostas espectrais e temporais diferentes.</x:v>
       </x:c>
@@ -4674,10 +6423,10 @@
         <x:v>A especificação nominal não encerra a incerteza de campo.</x:v>
       </x:c>
       <x:c r="M31" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N31" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O31" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4698,7 +6447,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="32" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A32" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4714,7 +6463,9 @@
       <x:c r="E32" s="13" t="str">
         <x:v>cap. 3-7</x:v>
       </x:c>
-      <x:c r="F32" s="13" t="str"/>
+      <x:c r="F32" s="13" t="str">
+        <x:v>circumsolar region</x:v>
+      </x:c>
       <x:c r="G32" s="13" t="str">
         <x:v>Pireliômetros requerem alinhamento com o Sol e possuem campo de visão limitado.</x:v>
       </x:c>
@@ -4734,10 +6485,10 @@
         <x:v>Inclui uma região circumsolar conforme o instrumento.</x:v>
       </x:c>
       <x:c r="M32" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N32" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O32" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4758,7 +6509,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="33" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A33" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4774,7 +6525,9 @@
       <x:c r="E33" s="13" t="str">
         <x:v>cap. 4-1</x:v>
       </x:c>
-      <x:c r="F33" s="13" t="str"/>
+      <x:c r="F33" s="13" t="str">
+        <x:v>flagging suspicious or erroneous data</x:v>
+      </x:c>
       <x:c r="G33" s="13" t="str">
         <x:v>Avaliação e controle de qualidade tratam dados suspeitos e realimentam a operação.</x:v>
       </x:c>
@@ -4794,10 +6547,10 @@
         <x:v>Completude não é sinônimo de exatidão.</x:v>
       </x:c>
       <x:c r="M33" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N33" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O33" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4818,7 +6571,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="34" ht="84" hidden="0" customHeight="1">
       <x:c r="A34" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4834,7 +6587,9 @@
       <x:c r="E34" s="13" t="str">
         <x:v>cap. 4-15</x:v>
       </x:c>
-      <x:c r="F34" s="13" t="str"/>
+      <x:c r="F34" s="13" t="str">
+        <x:v>especially when only a single radiometer exists locally</x:v>
+      </x:c>
       <x:c r="G34" s="13" t="str">
         <x:v>Uma única medição inclinada impõe limitações ao controle de qualidade radiométrico.</x:v>
       </x:c>
@@ -4854,10 +6609,10 @@
         <x:v>Ausência de referências independentes limita o diagnóstico.</x:v>
       </x:c>
       <x:c r="M34" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre definições radiométricas, Tabela 3-1, resposta do instrumento e limitações de QC do cap. 4; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N34" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O34" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4878,7 +6633,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="35" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A35" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4894,7 +6649,9 @@
       <x:c r="E35" s="13" t="str">
         <x:v>cap. 7-1</x:v>
       </x:c>
-      <x:c r="F35" s="13" t="str"/>
+      <x:c r="F35" s="13" t="str">
+        <x:v>Site-adaptation models have been used</x:v>
+      </x:c>
       <x:c r="G35" s="13" t="str">
         <x:v>Modelos de satélite e adaptação local ampliam a caracterização do recurso.</x:v>
       </x:c>
@@ -4914,10 +6671,10 @@
         <x:v>Irradiância de superfície é saída de modelagem.</x:v>
       </x:c>
       <x:c r="M35" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N35" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O35" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4938,7 +6695,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="36" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A36" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -4954,7 +6711,9 @@
       <x:c r="E36" s="13" t="str">
         <x:v>cap. 7-2</x:v>
       </x:c>
-      <x:c r="F36" s="13" t="str"/>
+      <x:c r="F36" s="13" t="str">
+        <x:v>reanalysis mode for historical time series</x:v>
+      </x:c>
       <x:c r="G36" s="13" t="str">
         <x:v>Reanálises produzem séries históricas de GHI a partir de sistemas atmosféricos.</x:v>
       </x:c>
@@ -4974,10 +6733,10 @@
         <x:v>Não representam estações radiométricas em cada ponto.</x:v>
       </x:c>
       <x:c r="M36" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N36" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O36" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -4998,7 +6757,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="37" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A37" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -5014,7 +6773,9 @@
       <x:c r="E37" s="13" t="str">
         <x:v>cap. 7-8</x:v>
       </x:c>
-      <x:c r="F37" s="13" t="str"/>
+      <x:c r="F37" s="13" t="str">
+        <x:v>derives cloud optical properties</x:v>
+      </x:c>
       <x:c r="G37" s="13" t="str">
         <x:v>Modelos físicos de satélite podem recuperar nuvens e usar transferência radiativa.</x:v>
       </x:c>
@@ -5034,10 +6795,10 @@
         <x:v>Não tratar a estimativa superficial como leitura direta do sensor orbital.</x:v>
       </x:c>
       <x:c r="M37" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N37" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA</x:v>
       </x:c>
       <x:c r="O37" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -5058,7 +6819,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="38" ht="84" hidden="0" customHeight="1">
       <x:c r="A38" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -5074,7 +6835,9 @@
       <x:c r="E38" s="13" t="str">
         <x:v>cap. 8-4</x:v>
       </x:c>
-      <x:c r="F38" s="13" t="str"/>
+      <x:c r="F38" s="13" t="str">
+        <x:v>TMY data are not designed to provide meteorological extremes</x:v>
+      </x:c>
       <x:c r="G38" s="13" t="str">
         <x:v>Um ano meteorológico típico é uma construção estatística com finalidade própria.</x:v>
       </x:c>
@@ -5094,10 +6857,10 @@
         <x:v>Não reconstitui um período histórico específico nem preserva todos os extremos.</x:v>
       </x:c>
       <x:c r="M38" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N38" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O38" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -5118,7 +6881,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="39" ht="84" hidden="0" customHeight="1">
       <x:c r="A39" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -5134,7 +6897,9 @@
       <x:c r="E39" s="13" t="str">
         <x:v>cap. 10-5</x:v>
       </x:c>
-      <x:c r="F39" s="13" t="str"/>
+      <x:c r="F39" s="13" t="str">
+        <x:v>the measurand has four general sources of uncertainty</x:v>
+      </x:c>
       <x:c r="G39" s="13" t="str">
         <x:v>Incerteza depende do mensurando e de contribuições da medição e da calibração.</x:v>
       </x:c>
@@ -5154,10 +6919,10 @@
         <x:v>Uma métrica de erro não resume toda a incerteza.</x:v>
       </x:c>
       <x:c r="M39" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N39" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O39" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -5178,7 +6943,7 @@
         <x:v>Não</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="33.599998474121094" hidden="0" customHeight="1">
+    <x:row r="40" ht="67.19999694824219" hidden="0" customHeight="1">
       <x:c r="A40" s="13" t="str">
         <x:v>1.4</x:v>
       </x:c>
@@ -5194,7 +6959,9 @@
       <x:c r="E40" s="13" t="str">
         <x:v>cap. 10-6</x:v>
       </x:c>
-      <x:c r="F40" s="13" t="str"/>
+      <x:c r="F40" s="13" t="str">
+        <x:v>uncertainty in its input data</x:v>
+      </x:c>
       <x:c r="G40" s="13" t="str">
         <x:v>Modelos, entradas, propagação e referência contribuem para a incerteza estimada.</x:v>
       </x:c>
@@ -5214,10 +6981,10 @@
         <x:v>Contribuições podem depender do local e período.</x:v>
       </x:c>
       <x:c r="M40" s="13" t="str">
-        <x:v>Localizadores conferidos</x:v>
+        <x:v>Comparação entre métodos do cap. 7, representatividade/TMY do cap. 8 e fontes de incerteza do cap. 10; mesma coletânea.</x:v>
       </x:c>
       <x:c r="N40" s="13" t="str">
-        <x:v>Conferida em leitura localizada</x:v>
+        <x:v>DIRETA_COM_RESTRICAO</x:v>
       </x:c>
       <x:c r="O40" s="13" t="str">
         <x:v>https://docs.nrel.gov/docs/fy24osti/88300.pdf</x:v>
@@ -5241,7 +7008,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f2ca3fdb29545d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re72a79a641224bf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5281,7 +7048,7 @@
         <x:v>Não citar páginas de edição não consultada.</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>Pendente; não usada como prova</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
@@ -5295,7 +7062,7 @@
         <x:v>A034 só pode ser citado com seus dados reais.</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Pendente; não usada como prova</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45" customHeight="1">
@@ -5309,7 +7076,7 @@
         <x:v>Referência deve corresponder ao arquivo efetivamente lido.</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Verificar citação</x:v>
+        <x:v>não selecionada como prova; PDF disponível com fontes e recursos gráficos danificados; 4ª edição lida separadamente</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="45" customHeight="1">
@@ -5323,7 +7090,7 @@
         <x:v>Não apresentar inversões como observação.</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
-        <x:v>Restrição metodológica</x:v>
+        <x:v>dados preparados conferidos; citação DOI confirmada em material DOE/NREL, p. 25</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
@@ -5414,14 +7181,16 @@
         <x:v>2024</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>complementar; foco em transposição da subseção 3.1; leitura pendente</x:v>
+        <x:v>complementar selecionada; pp. 1 e 9–11 conferidas; limites da validação inversa</x:v>
       </x:c>
       <x:c r="E2" s="13" t="str">
         <x:v>PDF disponível</x:v>
       </x:c>
-      <x:c r="F2" s="13" t="str"/>
+      <x:c r="F2" s="13" t="str">
+        <x:v>1,9,10,11</x:v>
+      </x:c>
       <x:c r="G2" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>fundamento de afirmações verificadas</x:v>
       </x:c>
       <x:c r="H2" s="13" t="str">
         <x:v>Modelo de céu e componentes para transposição.</x:v>
@@ -5459,7 +7228,7 @@
         <x:v>https://doi.org/10.1002/9781119540328</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="16.799999237060547" hidden="0" customHeight="1">
+    <x:row r="4" ht="33.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="13" t="str">
         <x:v>B19</x:v>
       </x:c>
@@ -5470,14 +7239,14 @@
         <x:v>2ª edição, 2014</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
-        <x:v>pendente; edição exata ausente</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="E4" s="13" t="str">
         <x:v>PDF da edição exata NÃO localizado</x:v>
       </x:c>
       <x:c r="F4" s="13" t="str"/>
       <x:c r="G4" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="H4" s="13" t="str">
         <x:v>Não substituir silenciosamente por A003.</x:v>
@@ -5486,7 +7255,7 @@
         <x:v>https://doi.org/10.1016/c2011-0-07038-2</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="16.799999237060547" hidden="0" customHeight="1">
+    <x:row r="5" ht="33.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" s="13" t="str">
         <x:v>B20</x:v>
       </x:c>
@@ -5497,14 +7266,14 @@
         <x:v>2ª edição, 2011</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
-        <x:v>pendente; edição exata ausente</x:v>
+        <x:v>não selecionada como prova desta versão; edição exata ausente no recorte inspecionado</x:v>
       </x:c>
       <x:c r="E5" s="13" t="str">
         <x:v>PDF da 2ª edição NÃO localizado</x:v>
       </x:c>
       <x:c r="F5" s="13" t="str"/>
       <x:c r="G5" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="H5" s="13" t="str">
         <x:v>A034 é a 1ª edição de 2003, apenas apoio.</x:v>
@@ -5553,14 +7322,14 @@
         <x:v>Conjunto publicado em 2021; observações de 2024</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>dados preparados conferidos; metadados DOI herdados</x:v>
+        <x:v>dados preparados conferidos; citação DOI confirmada em material DOE/NREL, p. 25</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
         <x:v>Conjunto de dados online</x:v>
       </x:c>
       <x:c r="F7" s="13" t="str"/>
       <x:c r="G7" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="H7" s="13" t="str">
         <x:v>Dados de campo POA/geração; sem GHI/DNI/DHI locais medidos.</x:v>
@@ -5587,7 +7356,7 @@
       </x:c>
       <x:c r="F8" s="13" t="str"/>
       <x:c r="G8" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
         <x:v>Contextualização do Farm Solar Array e do tratamento de dados.</x:v>
@@ -5596,7 +7365,7 @@
         <x:v>https://pv-tutorials.github.io/2024_Analytics_Webinar/solar-data-tools-demo.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="16.799999237060547" hidden="0" customHeight="1">
+    <x:row r="9" ht="33.599998474121094" hidden="0" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>B27</x:v>
       </x:c>
@@ -5607,14 +7376,14 @@
         <x:v>Versão online</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>documentação catalogada; leitura pendente</x:v>
+        <x:v>README oficial conferido; proveniência e acesso; sem presumir leitura de todo o acervo</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
         <x:v>Repositório/documentação online</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str"/>
       <x:c r="G9" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="H9" s="13" t="str">
         <x:v>Acesso e proveniência técnica do conjunto de dados.</x:v>
@@ -5719,14 +7488,16 @@
         <x:v>IEA PVPS T16-04:2021</x:v>
       </x:c>
       <x:c r="D13" s="13" t="str">
-        <x:v>PDF da 3ª edição disponível; leitura pendente; não confundir com A045/2024</x:v>
+        <x:v>não selecionada como prova; PDF disponível com fontes e recursos gráficos danificados; 4ª edição lida separadamente</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
         <x:v>PDF disponível nas pastas 1.2–1.4</x:v>
       </x:c>
-      <x:c r="F13" s="13" t="str"/>
+      <x:c r="F13" s="13" t="str">
+        <x:v>26,28,29,55</x:v>
+      </x:c>
       <x:c r="G13" s="13" t="str">
-        <x:v>complemento/contexto/pendência</x:v>
+        <x:v>proveniência/contexto/decisão de exclusão</x:v>
       </x:c>
       <x:c r="H13" s="13" t="str">
         <x:v>PDF consultado é o formato IEA PVPS; DOI aponta para o formato NREL.</x:v>
@@ -5792,7 +7563,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f332fd1a8b84fde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd8f27ea77044547"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>